<commit_message>
Added the code with Threading for Multiple session run parallel, changed prompt directory
</commit_message>
<xml_diff>
--- a/backend/session_data/sessions.xlsx
+++ b/backend/session_data/sessions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,6 +549,16 @@
           <t>current_step</t>
         </is>
       </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>thread_id</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>thread_name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -655,6 +665,8 @@
           <t>Workflow completed</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -761,6 +773,8 @@
           <t>Workflow completed</t>
         </is>
       </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -867,6 +881,8 @@
           <t>Workflow completed</t>
         </is>
       </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -973,6 +989,8 @@
           <t>Workflow completed</t>
         </is>
       </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1079,6 +1097,8 @@
           <t>Workflow completed</t>
         </is>
       </c>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1183,6 +1203,1614 @@
       <c r="X7" t="inlineStr">
         <is>
           <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:02:34.400997</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:02:57.043071</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:02:57.043071</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa_code.py</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_02_34__d94f9b4d-6dac-4aff-a739-1f09a11a9aaa_summary.md</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>dump() missing 1 required positional argument: 'fp'</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traceback (most recent call last):
+  File "E:\AI\Projects\Agentic-AI-Based-AutoML-Application\backend\thread_main.py", line 259, in run_ml_workflow_sync
+    json.dump(results, default=make_json_safe, indent=2)
+TypeError: dump() missing 1 required positional argument: 'fp'
+</t>
+        </is>
+      </c>
+      <c r="W8" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>21772</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:04:34.554711</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:04:48.477179</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:04:48.433513</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829_code.py</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829_summary.md</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_04_34__486f1bf1-0bec-4d1c-9e63-eb356bd1d829_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:05:21.943418</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:05:37.726206</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:05:37.685458</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a_code.py</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a_summary.md</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_05_21__96189076-272e-4dd3-bf70-95e74eef7a3a_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>1</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:06:10.206706</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:06:22.734920</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:06:22.691322</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7_code.py</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7_summary.md</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_06_10__e496b6aa-e054-4067-888e-e9d75e4c24f7_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>1</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:11:35.412280</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:11:50.404257</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:11:50.360531</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b_code.py</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b_summary.md</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_11_35__e6f029c9-21a6-4e5d-8079-d652f1097e2b_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:13:35.378715</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:13:48.661666</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:13:48.618484</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee_code.py</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee_summary.md</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_13_35__31186f02-c102-4159-b380-2b0da450d6ee_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="n">
+        <v>1</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:16:27.935122</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:16:52.066929</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:16:52.011468</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929_code.py</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929_summary.md</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_16_27__c51b2007-43a6-48e9-bab8-892e183d8929_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:23:47.385499</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:24:02.529087</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:24:02.499121</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d_code.py</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d_summary.md</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_23_47__c41d1bab-e87e-4faf-bcaf-26fa1eacab2d_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>1</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:32:25.171984</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:32:41.290158</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:32:41.241847</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3_code.py</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3_summary.md</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_32_25__8cb4800d-18f2-4411-a2d4-ef66714cfbe3_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="n">
+        <v>1</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y16" t="n">
+        <v>18876</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:37:27.732743</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:37:50.910449</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:37:50.841420</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b_code.py</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b_summary.md</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_37_27__12ac8903-a79e-4c5c-a1f6-6e3307302a3b_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>1</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y17" t="n">
+        <v>13060</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd_Churn_Modelling.csv</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:37:29.784946</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:37:52.480074</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:37:52.427022</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd_code.py</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd_summary.md</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_37_29__ecc1dab1-2a3a-4f12-851c-daabb399cebd_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="n">
+        <v>1</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>1812</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>MLWorkflow_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>synthetic_coffee_health_10000.csv</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b_synthetic_coffee_health_10000.csv</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Alcohol_Consumption</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:40:07.020144</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:40:27.689548</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:40:27.639276</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b_code.py</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b_summary.md</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_40_07__7b4c7c8a-b2b9-4ec5-8742-01547dbaf39b_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="n">
+        <v>1</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y19" t="n">
+        <v>13060</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>wine_quality_merged.csv</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426_wine_quality_merged.csv</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:40:09.126341</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:40:24.107979</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2025-11-01T10:40:23.979735</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426_code.py</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426_summary.md</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__10_40_09__b6c3f96e-f715-42d7-b7e8-bbadd95f1426_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>XGBClassifier</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>1</v>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>1812</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>MLWorkflow_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>synthetic_coffee_health_10000.csv</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>uploads/2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999_synthetic_coffee_health_10000.csv</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Alcohol_Consumption</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2025-11-01T11:01:20.443692</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2025-11-01T11:01:39.207800</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2025-11-01T11:01:39.164527</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>generated_code/2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999_code.py</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>results/2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999_classification_results.json</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>model/2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999_classification_models.zip</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>ai_summary/2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999_summary.md</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>workflow_info/2025_11_01__11_01_20__03755142-8d13-4bd9-8c96-cb48b4ed5999_workflow_results.json</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>classification</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>1</v>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Workflow completed</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>22048</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>MLWorkflow_0</t>
         </is>
       </c>
     </row>

</xml_diff>